<commit_message>
Revert unnecessary API mapping rows
</commit_message>
<xml_diff>
--- a/torch_to_mindspore_mapping.xlsx
+++ b/torch_to_mindspore_mapping.xlsx
@@ -14867,16 +14867,6 @@
       <c r="C842" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D842" t="inlineStr">
-        <is>
-          <t>mindspore.ops.flash_attention_score; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E842" t="inlineStr">
-        <is>
-          <t>参数和 layout 有差异; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
     </row>
     <row r="843" ht="16" customHeight="1">
       <c r="A843" s="1" t="inlineStr">
@@ -14917,18 +14907,7 @@
       <c r="C846" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D846" s="12" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.grouped_matmul; 
-mindspore.ops.auto_generate.grouped_matmul_v2; 
-mindspore.ops.auto_generate.grouped_matmul_v4; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E846" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；Ascend 融合算子，参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="D846" s="12" t="n"/>
     </row>
     <row r="847" ht="16" customHeight="1">
       <c r="A847" s="1" t="inlineStr">
@@ -15006,23 +14985,8 @@
           <t>torch_npu.npu_rms_norm</t>
         </is>
       </c>
-      <c r="B853" t="inlineStr">
-        <is>
-          <t>mindspore.ops.rms_norm</t>
-        </is>
-      </c>
       <c r="C853" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="D853" t="inlineStr">
-        <is>
-          <t>hyper_parallel.models.modules.rmsnorm.RMSNorm</t>
-        </is>
-      </c>
-      <c r="E853" t="inlineStr">
-        <is>
-          <t>hyper-parallel 有 RMSNorm eager fallback/fused path 可参考</t>
-        </is>
       </c>
     </row>
     <row r="854" ht="16" customHeight="1">
@@ -15044,16 +15008,6 @@
       <c r="C855" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D855" t="inlineStr">
-        <is>
-          <t>mindspore.ops.rotary_position_embedding; hyper_parallel.models.modules.rope.apply_rotary_pos_emb; hyper_parallel.models.modules.rope.MultiModalRotaryEmbedding</t>
-        </is>
-      </c>
-      <c r="E855" t="inlineStr">
-        <is>
-          <t>rotary_mul 与 rotary_position_embedding 参数语义不同; hyper-parallel 有 RoPE/mRoPE 手写实现可参考，适合替代 rotary 类私有融合算子但需核对 shape/layout</t>
-        </is>
-      </c>
     </row>
     <row r="856" hidden="1" ht="16" customHeight="1">
       <c r="A856" s="1" t="inlineStr">
@@ -15061,23 +15015,8 @@
           <t>torch_npu.npu_swiglu</t>
         </is>
       </c>
-      <c r="B856" t="inlineStr">
-        <is>
-          <t>mindspore.ops.swiglu</t>
-        </is>
-      </c>
       <c r="C856" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="D856" t="inlineStr">
-        <is>
-          <t>hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E856" t="inlineStr">
-        <is>
-          <t>hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
       </c>
     </row>
     <row r="857" hidden="1" ht="16" customHeight="1">
@@ -15576,149 +15515,32 @@
       </c>
     </row>
     <row r="894" hidden="1" ht="16.8" customHeight="1">
-      <c r="A894" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="B894" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="C894" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D894" t="inlineStr">
-        <is>
-          <t>mindspore.ops.speed_fusion_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E894" t="inlineStr">
-        <is>
-          <t>推理融合注意力公开接口，参数和 layout 需核对; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A894" s="1" t="n"/>
+      <c r="C894" s="5" t="n"/>
     </row>
     <row r="895" hidden="1" ht="16.8" customHeight="1">
-      <c r="A895" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_grouped_matmul_finalize_routing</t>
-        </is>
-      </c>
-      <c r="C895" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D895" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.grouped_matmul; mindspore.ops.auto_generate.moe_finalize_routing; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E895" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；未找到单一对等接口，可拆分替代; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A895" s="1" t="n"/>
+      <c r="C895" s="5" t="n"/>
     </row>
     <row r="896" hidden="1" ht="16.8" customHeight="1">
-      <c r="A896" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_distribute_combine_v2</t>
-        </is>
-      </c>
-      <c r="C896" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D896" t="inlineStr">
-        <is>
-          <t>mindspore.ops.moe_distribute_combine; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E896" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；v2/参数可能不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A896" s="1" t="n"/>
+      <c r="C896" s="5" t="n"/>
     </row>
     <row r="897" hidden="1" ht="16.8" customHeight="1">
-      <c r="A897" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_distribute_dispatch_v2</t>
-        </is>
-      </c>
-      <c r="C897" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D897" t="inlineStr">
-        <is>
-          <t>mindspore.ops.moe_distribute_dispatch; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E897" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；v2/参数可能不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A897" s="1" t="n"/>
+      <c r="C897" s="5" t="n"/>
     </row>
     <row r="898" hidden="1" ht="16.8" customHeight="1">
-      <c r="A898" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_finalize_routing</t>
-        </is>
-      </c>
-      <c r="C898" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D898" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.moe_finalize_routing; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E898" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A898" s="1" t="n"/>
+      <c r="C898" s="5" t="n"/>
     </row>
     <row r="899" hidden="1" ht="16.8" customHeight="1">
-      <c r="A899" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_gating_top_k</t>
-        </is>
-      </c>
-      <c r="C899" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D899" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.moe_gating_top_k_softmax; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E899" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；包含 softmax/top-k 语义，参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A899" s="1" t="n"/>
+      <c r="C899" s="5" t="n"/>
     </row>
     <row r="900" hidden="1" ht="16.8" customHeight="1">
-      <c r="A900" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_init_routing_v2</t>
-        </is>
-      </c>
-      <c r="C900" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D900" t="inlineStr">
-        <is>
-          <t>mindspore.ops.moe_init_routing_v2; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E900" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A900" s="1" t="n"/>
+      <c r="C900" s="5" t="n"/>
     </row>
     <row r="901" hidden="1" ht="16.8" customHeight="1">
       <c r="A901" s="1" t="inlineStr">
@@ -16481,24 +16303,8 @@
       </c>
     </row>
     <row r="949" hidden="1" ht="16.8" customHeight="1">
-      <c r="A949" s="1" t="inlineStr">
-        <is>
-          <t>torch.ops.custom.npu_ai_infra_kv_quant_sparse_flash_attention</t>
-        </is>
-      </c>
-      <c r="C949" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D949" t="inlineStr">
-        <is>
-          <t>mindspore.ops.sparse_flash_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E949" t="inlineStr">
-        <is>
-          <t>自定义接口，KV quant 参数需人工核对; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A949" s="1" t="n"/>
+      <c r="C949" s="5" t="n"/>
     </row>
     <row r="950" ht="16.8" customHeight="1">
       <c r="A950" s="1" t="inlineStr">
@@ -16521,24 +16327,8 @@
       </c>
     </row>
     <row r="952" hidden="1" ht="16.8" customHeight="1">
-      <c r="A952" s="1" t="inlineStr">
-        <is>
-          <t>torch.ops.custom.npu_ai_infra_sparse_flash_attention_pioneer</t>
-        </is>
-      </c>
-      <c r="C952" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D952" t="inlineStr">
-        <is>
-          <t>mindspore.ops.sparse_flash_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E952" t="inlineStr">
-        <is>
-          <t>自定义接口，参数需人工核对; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A952" s="1" t="n"/>
+      <c r="C952" s="5" t="n"/>
     </row>
     <row r="953" hidden="1" ht="16.8" customHeight="1">
       <c r="A953" s="1" t="inlineStr">
@@ -16581,29 +16371,8 @@
       </c>
     </row>
     <row r="955" hidden="1" ht="16.8" customHeight="1">
-      <c r="A955" s="1" t="inlineStr">
-        <is>
-          <t>torch.ops.npu.npu_fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="B955" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="C955" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D955" t="inlineStr">
-        <is>
-          <t>mindspore.ops.speed_fusion_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E955" t="inlineStr">
-        <is>
-          <t>参数和 layout 需核对; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A955" s="1" t="n"/>
+      <c r="C955" s="5" t="n"/>
     </row>
     <row r="956" ht="16.8" customHeight="1">
       <c r="A956" s="1" t="inlineStr">
@@ -16716,44 +16485,12 @@
       </c>
     </row>
     <row r="964" hidden="1" ht="16.8" customHeight="1">
-      <c r="A964" s="1" t="inlineStr">
-        <is>
-          <t>torch.ops.vllm.unified_attention</t>
-        </is>
-      </c>
-      <c r="C964" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D964" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score; mindspore.ops.flash_attention_score; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E964" t="inlineStr">
-        <is>
-          <t>vLLM 自定义接口，需按注意力场景改写; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A964" s="1" t="n"/>
+      <c r="C964" s="5" t="n"/>
     </row>
     <row r="965" hidden="1" ht="16.8" customHeight="1">
-      <c r="A965" s="1" t="inlineStr">
-        <is>
-          <t>torch.ops.vllm.unified_attention_with_output</t>
-        </is>
-      </c>
-      <c r="C965" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D965" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score; mindspore.ops.flash_attention_score; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E965" t="inlineStr">
-        <is>
-          <t>vLLM 自定义接口，需按注意力场景改写; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A965" s="1" t="n"/>
+      <c r="C965" s="5" t="n"/>
     </row>
     <row r="966" hidden="1" ht="16.8" customHeight="1">
       <c r="A966" s="1" t="inlineStr">
@@ -17326,49 +17063,12 @@
       </c>
     </row>
     <row r="1006" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1006" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_add_rms_norm</t>
-        </is>
-      </c>
-      <c r="B1006" t="inlineStr">
-        <is>
-          <t>mindspore.ops.add_rms_norm</t>
-        </is>
-      </c>
-      <c r="C1006" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1006" t="inlineStr">
-        <is>
-          <t>hyper_parallel.models.modules.rmsnorm.RMSNormGated</t>
-        </is>
-      </c>
-      <c r="E1006" t="inlineStr">
-        <is>
-          <t>hyper-parallel 有 gated RMSNorm 组合实现可参考，但不等价于 add_rms_norm 融合接口</t>
-        </is>
-      </c>
+      <c r="A1006" s="1" t="n"/>
+      <c r="C1006" s="5" t="n"/>
     </row>
     <row r="1007" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1007" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_apply_rotary_pos_emb</t>
-        </is>
-      </c>
-      <c r="C1007" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1007" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.apply_rotary_pos_emb; mindspore.ops.rotary_position_embedding; hyper_parallel.models.modules.rope.apply_rotary_pos_emb; hyper_parallel.models.modules.rope.MultiModalRotaryEmbedding</t>
-        </is>
-      </c>
-      <c r="E1007" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；参数语义需人工核对; hyper-parallel 有 RoPE/mRoPE 手写实现可参考，适合替代 rotary 类私有融合算子但需核对 shape/layout</t>
-        </is>
-      </c>
+      <c r="A1007" s="1" t="n"/>
+      <c r="C1007" s="5" t="n"/>
     </row>
     <row r="1008" ht="16.8" customHeight="1">
       <c r="A1008" s="1" t="inlineStr">
@@ -17421,99 +17121,20 @@
       </c>
     </row>
     <row r="1012" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1012" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_fused_infer_attention_score.out</t>
-        </is>
-      </c>
-      <c r="B1012" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="C1012" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1012" t="inlineStr">
-        <is>
-          <t>mindspore.ops.speed_fusion_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E1012" t="inlineStr">
-        <is>
-          <t>out 变体需改写为普通返回值; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A1012" s="1" t="n"/>
+      <c r="C1012" s="5" t="n"/>
     </row>
     <row r="1013" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1013" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_fused_infer_attention_score_v2</t>
-        </is>
-      </c>
-      <c r="B1013" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="C1013" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1013" t="inlineStr">
-        <is>
-          <t>mindspore.ops.speed_fusion_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E1013" t="inlineStr">
-        <is>
-          <t>v2 参数和 layout 需核对; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A1013" s="1" t="n"/>
+      <c r="C1013" s="5" t="n"/>
     </row>
     <row r="1014" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1014" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_fused_infer_attention_score_v2.out</t>
-        </is>
-      </c>
-      <c r="B1014" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="C1014" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1014" t="inlineStr">
-        <is>
-          <t>mindspore.ops.speed_fusion_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E1014" t="inlineStr">
-        <is>
-          <t>out/v2 变体需改写为普通返回值; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A1014" s="1" t="n"/>
+      <c r="C1014" s="5" t="n"/>
     </row>
     <row r="1015" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1015" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_interleave_rope</t>
-        </is>
-      </c>
-      <c r="C1015" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1015" t="inlineStr">
-        <is>
-          <t>mindspore.ops.rotary_position_embedding; hyper_parallel.models.modules.rope.apply_rotary_pos_emb; hyper_parallel.models.modules.rope.MultiModalRotaryEmbedding</t>
-        </is>
-      </c>
-      <c r="E1015" t="inlineStr">
-        <is>
-          <t>rotary/rope 类替代，参数不同; hyper-parallel 有 RoPE/mRoPE 手写实现可参考，适合替代 rotary 类私有融合算子但需核对 shape/layout</t>
-        </is>
-      </c>
+      <c r="A1015" s="1" t="n"/>
+      <c r="C1015" s="5" t="n"/>
     </row>
     <row r="1016" ht="16.8" customHeight="1">
       <c r="A1016" s="1" t="inlineStr">
@@ -17576,84 +17197,20 @@
       </c>
     </row>
     <row r="1022" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1022" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_compute_expert_tokens</t>
-        </is>
-      </c>
-      <c r="C1022" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1022" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.moe_compute_expert_tokens; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E1022" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A1022" s="1" t="n"/>
+      <c r="C1022" s="5" t="n"/>
     </row>
     <row r="1023" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1023" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_gating_top_k_softmax</t>
-        </is>
-      </c>
-      <c r="C1023" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1023" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.moe_gating_top_k_softmax; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E1023" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A1023" s="1" t="n"/>
+      <c r="C1023" s="5" t="n"/>
     </row>
     <row r="1024" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1024" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_moe_init_routing</t>
-        </is>
-      </c>
-      <c r="C1024" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1024" t="inlineStr">
-        <is>
-          <t>mindspore.ops.auto_generate.moe_init_routing; mindspore.ops.moe_init_routing_v2; hyper_parallel.platform.mindspore.multicore.moe_ffn_fwd/moe_ffn_bwd; hyper_parallel.platform.torch.common.moe.GroupedExperts</t>
-        </is>
-      </c>
-      <c r="E1024" t="inlineStr">
-        <is>
-          <t>代码已有，未对外；参数不同; hyper-parallel 有 MoE FFN/GroupedMatmul/SwiGLU 融合路径可参考，需按 omniinfer routing/tiling/workspace 参数人工适配</t>
-        </is>
-      </c>
+      <c r="A1024" s="1" t="n"/>
+      <c r="C1024" s="5" t="n"/>
     </row>
     <row r="1025" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1025" s="1" t="inlineStr">
-        <is>
-          <t>torch_npu.npu_mrope</t>
-        </is>
-      </c>
-      <c r="C1025" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1025" t="inlineStr">
-        <is>
-          <t>mindspore.ops.rotary_position_embedding; hyper_parallel.models.modules.rope.apply_rotary_pos_emb; hyper_parallel.models.modules.rope.MultiModalRotaryEmbedding</t>
-        </is>
-      </c>
-      <c r="E1025" t="inlineStr">
-        <is>
-          <t>mrope 需按多模态 rope 语义人工改写; hyper-parallel 有 RoPE/mRoPE 手写实现可参考，适合替代 rotary 类私有融合算子但需核对 shape/layout</t>
-        </is>
-      </c>
+      <c r="A1025" s="1" t="n"/>
+      <c r="C1025" s="5" t="n"/>
     </row>
     <row r="1026" ht="16.8" customHeight="1">
       <c r="A1026" s="1" t="inlineStr">
@@ -17776,29 +17333,8 @@
       </c>
     </row>
     <row r="1036" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1036" s="1" t="inlineStr">
-        <is>
-          <t>torchair.ops.npu_fused_infer_attention_score_v2</t>
-        </is>
-      </c>
-      <c r="B1036" t="inlineStr">
-        <is>
-          <t>mindspore.ops.fused_infer_attention_score</t>
-        </is>
-      </c>
-      <c r="C1036" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1036" t="inlineStr">
-        <is>
-          <t>mindspore.ops.speed_fusion_attention; hyper_parallel.core.shard.ops.parallel_npu_flash_attention_score.NPUFlashAttentionScoreDistributedOp</t>
-        </is>
-      </c>
-      <c r="E1036" t="inlineStr">
-        <is>
-          <t>torchair 编译后端接口，迁移时改用 MindSpore 原生接口; hyper-parallel 可参考分布式 npu_fusion_attention 封装和 layout/sharding 测试，不是直接 MindSpore 公共 API</t>
-        </is>
-      </c>
+      <c r="A1036" s="1" t="n"/>
+      <c r="C1036" s="5" t="n"/>
     </row>
     <row r="1037" ht="16.8" customHeight="1">
       <c r="A1037" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Fix reverted API mapping rows
</commit_message>
<xml_diff>
--- a/torch_to_mindspore_mapping.xlsx
+++ b/torch_to_mindspore_mapping.xlsx
@@ -1934,13 +1934,22 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>mindspore.device_context.cpu/gpu/ascend.device_count</t>
+          <t>mindspore.device_context.gpu.device_count</t>
         </is>
       </c>
       <c r="C48" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="4" t="n"/>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>mindspore.device_context.cpu.device_count; mindspore.device_context.ascend.device_count</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>原写法 mindspore.device_context.cpu/gpu/ascend.device_count 不是有效 API；CUDA 场景优先对应 GPU</t>
+        </is>
+      </c>
     </row>
     <row r="49" hidden="1" ht="16" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -1990,14 +1999,22 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>mindspore.device_context.cpu/gpu/ascend.is_available</t>
+          <t>mindspore.device_context.gpu.is_available</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="9" t="n"/>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>mindspore.device_context.cpu.is_available; mindspore.device_context.ascend.is_available</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>原写法 mindspore.device_context.cpu/gpu/ascend.is_available 不是有效 API；CUDA 场景优先对应 GPU</t>
+        </is>
+      </c>
     </row>
     <row r="52" hidden="1" ht="16" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
@@ -3266,15 +3283,20 @@
           <t>torch.is_tensor</t>
         </is>
       </c>
-      <c r="B121" s="4" t="inlineStr">
-        <is>
-          <t>mindspore.is_tensor</t>
-        </is>
-      </c>
+      <c r="B121" s="4" t="n"/>
       <c r="C121" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D121" s="4" t="n"/>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>isinstance(obj, mindspore.Tensor)</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>mindspore.is_tensor 已废弃，2.9.0 后将删除</t>
+        </is>
+      </c>
     </row>
     <row r="122" hidden="1" ht="16" customHeight="1">
       <c r="A122" s="4" t="inlineStr">
@@ -4293,7 +4315,7 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>mindspore.nn.DropOut3d</t>
+          <t>mindspore.nn.Dropout3d</t>
         </is>
       </c>
       <c r="C178" s="5" t="n">
@@ -5457,7 +5479,7 @@
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>mindspore.parallel.distributedDistributedDataParallel</t>
+          <t>mindspore.parallel.distributed.DistributedDataParallel</t>
         </is>
       </c>
       <c r="C243" s="5" t="n">
@@ -5869,17 +5891,18 @@
           <t>torch.no_grad</t>
         </is>
       </c>
-      <c r="B267" s="8" t="inlineStr">
+      <c r="B267" s="8" t="n"/>
+      <c r="C267" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D267" t="inlineStr">
         <is>
           <t>mindspore._no_grad</t>
         </is>
       </c>
-      <c r="C267" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>参考：https://www.hiascend.com/forum/thread-0289146760766805055-1-1.html</t>
+          <t>代码已有，未对外；参考：https://www.hiascend.com/forum/thread-0289146760766805055-1-1.html</t>
         </is>
       </c>
     </row>
@@ -8241,7 +8264,16 @@
       <c r="C408" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D408" s="4" t="n"/>
+      <c r="D408" s="4" t="inlineStr">
+        <is>
+          <t>mindspore.mint.where</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>最新文档提示 2.9.0 后 masked_fill_ 返回值将改为无显式返回；可按场景改写为 where</t>
+        </is>
+      </c>
     </row>
     <row r="409" hidden="1" ht="16" customHeight="1">
       <c r="A409" s="4" t="inlineStr">
@@ -9958,18 +9990,18 @@
           <t>torch_scatter.scatter_max</t>
         </is>
       </c>
-      <c r="B512" s="4" t="inlineStr">
+      <c r="B512" s="4" t="n"/>
+      <c r="C512" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D512" s="4" t="inlineStr">
         <is>
           <t>mindspore.ops.scatter_max</t>
         </is>
       </c>
-      <c r="C512" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D512" s="4" t="n"/>
       <c r="E512" s="8" t="inlineStr">
         <is>
-          <t>torch_scatter：https://pytorch-scatter.readthedocs.io/en/1.3.0/functions/max.html</t>
+          <t>torch_scatter：https://pytorch-scatter.readthedocs.io/en/1.3.0/functions/max.html；mindspore.ops.scatter_max 已废弃，2.9.0 后将删除，未找到公开非废弃对等接口</t>
         </is>
       </c>
     </row>
@@ -10525,13 +10557,17 @@
       </c>
       <c r="B549" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.current_stream</t>
+          <t>mindspore.runtime.current_stream</t>
         </is>
       </c>
       <c r="C549" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E549" s="2" t="n"/>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="550" hidden="1" ht="16" customHeight="1">
       <c r="A550" s="1" t="inlineStr">
@@ -10541,13 +10577,17 @@
       </c>
       <c r="B550" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.default_stream</t>
+          <t>mindspore.runtime.default_stream</t>
         </is>
       </c>
       <c r="C550" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E550" s="2" t="n"/>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="551" hidden="1" ht="16" customHeight="1">
       <c r="A551" s="1" t="inlineStr">
@@ -10652,13 +10692,17 @@
       </c>
       <c r="B556" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.max_memory_allocated</t>
+          <t>mindspore.runtime.max_memory_allocated</t>
         </is>
       </c>
       <c r="C556" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E556" s="2" t="n"/>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="557" hidden="1" ht="16" customHeight="1">
       <c r="A557" s="1" t="inlineStr">
@@ -10668,13 +10712,17 @@
       </c>
       <c r="B557" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.max_memory_reserved</t>
+          <t>mindspore.runtime.max_memory_reserved</t>
         </is>
       </c>
       <c r="C557" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E557" s="2" t="n"/>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="558" hidden="1" ht="16" customHeight="1">
       <c r="A558" s="1" t="inlineStr">
@@ -10684,13 +10732,17 @@
       </c>
       <c r="B558" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.memory_allocated</t>
+          <t>mindspore.runtime.memory_allocated</t>
         </is>
       </c>
       <c r="C558" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E558" s="2" t="n"/>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="559" hidden="1" ht="16" customHeight="1">
       <c r="A559" s="1" t="inlineStr">
@@ -10700,13 +10752,17 @@
       </c>
       <c r="B559" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.memory_reserved</t>
+          <t>mindspore.runtime.memory_reserved</t>
         </is>
       </c>
       <c r="C559" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E559" s="2" t="n"/>
+      <c r="E559" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="560" hidden="1" ht="16" customHeight="1">
       <c r="A560" s="1" t="inlineStr">
@@ -10716,13 +10772,17 @@
       </c>
       <c r="B560" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.memory_stats</t>
+          <t>mindspore.runtime.memory_stats</t>
         </is>
       </c>
       <c r="C560" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E560" s="2" t="n"/>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="561" hidden="1" ht="16" customHeight="1">
       <c r="A561" s="1" t="inlineStr">
@@ -10748,13 +10808,17 @@
       </c>
       <c r="B562" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.Stream</t>
+          <t>mindspore.runtime.Stream</t>
         </is>
       </c>
       <c r="C562" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E562" s="2" t="n"/>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="563" hidden="1" ht="16" customHeight="1">
       <c r="A563" s="1" t="inlineStr">
@@ -11469,13 +11533,17 @@
       </c>
       <c r="B605" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.current_stream</t>
+          <t>mindspore.runtime.current_stream</t>
         </is>
       </c>
       <c r="C605" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E605" s="2" t="n"/>
+      <c r="E605" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="606" hidden="1" ht="16" customHeight="1">
       <c r="A606" s="1" t="inlineStr">
@@ -11485,13 +11553,17 @@
       </c>
       <c r="B606" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.default_stream</t>
+          <t>mindspore.runtime.default_stream</t>
         </is>
       </c>
       <c r="C606" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E606" s="2" t="n"/>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="607" hidden="1" ht="16" customHeight="1">
       <c r="A607" s="1" t="inlineStr">
@@ -11501,13 +11573,22 @@
       </c>
       <c r="B607" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.device_count</t>
+          <t>mindspore.device_context.ascend.device_count</t>
         </is>
       </c>
       <c r="C607" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E607" s="2" t="n"/>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>mindspore.device_context.cpu.device_count; mindspore.device_context.gpu.device_count</t>
+        </is>
+      </c>
+      <c r="E607" s="2" t="inlineStr">
+        <is>
+          <t>mindspore.hal.device_count 已废弃；NPU 场景优先对应 ascend</t>
+        </is>
+      </c>
     </row>
     <row r="608" hidden="1" ht="16" customHeight="1">
       <c r="A608" s="1" t="inlineStr">
@@ -11517,13 +11598,17 @@
       </c>
       <c r="B608" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.empty_cache</t>
+          <t>mindspore.runtime.empty_cache</t>
         </is>
       </c>
       <c r="C608" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E608" s="2" t="n"/>
+      <c r="E608" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="609" hidden="1" ht="16" customHeight="1">
       <c r="A609" s="1" t="inlineStr">
@@ -11533,13 +11618,17 @@
       </c>
       <c r="B609" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.Event</t>
+          <t>mindspore.runtime.Event</t>
         </is>
       </c>
       <c r="C609" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E609" s="2" t="n"/>
+      <c r="E609" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="610" hidden="1" ht="16" customHeight="1">
       <c r="A610" s="1" t="inlineStr">
@@ -11549,13 +11638,22 @@
       </c>
       <c r="B610" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.is_available</t>
+          <t>mindspore.device_context.ascend.is_available</t>
         </is>
       </c>
       <c r="C610" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E610" s="2" t="n"/>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>mindspore.device_context.cpu.is_available; mindspore.device_context.gpu.is_available</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="inlineStr">
+        <is>
+          <t>mindspore.hal.is_available 已废弃；NPU 场景优先对应 ascend</t>
+        </is>
+      </c>
     </row>
     <row r="611" hidden="1" ht="16" customHeight="1">
       <c r="A611" s="1" t="inlineStr">
@@ -11565,13 +11663,17 @@
       </c>
       <c r="B611" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.max_memory_allocated</t>
+          <t>mindspore.runtime.max_memory_allocated</t>
         </is>
       </c>
       <c r="C611" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E611" s="2" t="n"/>
+      <c r="E611" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="612" hidden="1" ht="16" customHeight="1">
       <c r="A612" s="1" t="inlineStr">
@@ -11581,13 +11683,17 @@
       </c>
       <c r="B612" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.max_memory_reserved</t>
+          <t>mindspore.runtime.max_memory_reserved</t>
         </is>
       </c>
       <c r="C612" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E612" s="2" t="n"/>
+      <c r="E612" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="613" hidden="1" ht="16" customHeight="1">
       <c r="A613" s="1" t="inlineStr">
@@ -11597,13 +11703,17 @@
       </c>
       <c r="B613" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.memory_allocated</t>
+          <t>mindspore.runtime.memory_allocated</t>
         </is>
       </c>
       <c r="C613" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E613" s="2" t="n"/>
+      <c r="E613" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="614" hidden="1" ht="16" customHeight="1">
       <c r="A614" s="1" t="inlineStr">
@@ -11613,13 +11723,17 @@
       </c>
       <c r="B614" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.memory_reserved</t>
+          <t>mindspore.runtime.memory_reserved</t>
         </is>
       </c>
       <c r="C614" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E614" s="2" t="n"/>
+      <c r="E614" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="615" hidden="1" ht="16" customHeight="1">
       <c r="A615" s="1" t="inlineStr">
@@ -11629,13 +11743,17 @@
       </c>
       <c r="B615" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.memory_stats</t>
+          <t>mindspore.runtime.memory_stats</t>
         </is>
       </c>
       <c r="C615" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E615" s="2" t="n"/>
+      <c r="E615" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="616" hidden="1" ht="16" customHeight="1">
       <c r="A616" s="1" t="inlineStr">
@@ -11645,13 +11763,17 @@
       </c>
       <c r="B616" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.reset_peak_memory_stats</t>
+          <t>mindspore.runtime.reset_peak_memory_stats</t>
         </is>
       </c>
       <c r="C616" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E616" s="2" t="n"/>
+      <c r="E616" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="617" hidden="1" ht="16" customHeight="1">
       <c r="A617" s="1" t="inlineStr">
@@ -11677,13 +11799,17 @@
       </c>
       <c r="B618" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.Stream</t>
+          <t>mindspore.runtime.Stream</t>
         </is>
       </c>
       <c r="C618" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E618" s="2" t="n"/>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="619" hidden="1" ht="16" customHeight="1">
       <c r="A619" s="1" t="inlineStr">
@@ -11693,13 +11819,17 @@
       </c>
       <c r="B619" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.synchronize</t>
+          <t>mindspore.runtime.synchronize</t>
         </is>
       </c>
       <c r="C619" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E619" s="2" t="n"/>
+      <c r="E619" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="620" hidden="1" ht="16" customHeight="1">
       <c r="A620" s="1" t="inlineStr">
@@ -12567,13 +12697,17 @@
       </c>
       <c r="B672" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.current_stream</t>
+          <t>mindspore.runtime.current_stream</t>
         </is>
       </c>
       <c r="C672" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E672" s="2" t="n"/>
+      <c r="E672" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="673" hidden="1" ht="16" customHeight="1">
       <c r="A673" s="1" t="inlineStr">
@@ -12583,13 +12717,17 @@
       </c>
       <c r="B673" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.empty_cache</t>
+          <t>mindspore.runtime.empty_cache</t>
         </is>
       </c>
       <c r="C673" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E673" s="2" t="n"/>
+      <c r="E673" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="674" hidden="1" ht="16" customHeight="1">
       <c r="A674" s="1" t="inlineStr">
@@ -12599,13 +12737,17 @@
       </c>
       <c r="B674" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.Event</t>
+          <t>mindspore.runtime.Event</t>
         </is>
       </c>
       <c r="C674" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E674" s="2" t="n"/>
+      <c r="E674" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="675" hidden="1" ht="16" customHeight="1">
       <c r="A675" s="1" t="inlineStr">
@@ -12613,15 +12755,20 @@
           <t>torch_npu.npu.get_device_name</t>
         </is>
       </c>
-      <c r="B675" s="1" t="inlineStr">
+      <c r="B675" s="1" t="n"/>
+      <c r="C675" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D675" t="inlineStr">
         <is>
           <t>mindspore.hal.get_device_name</t>
         </is>
       </c>
-      <c r="C675" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E675" s="2" t="n"/>
+      <c r="E675" s="2" t="inlineStr">
+        <is>
+          <t>MindSpore 文档说明 hal.get_device_name 后续将废弃，未找到 runtime/device_context 公开对等接口</t>
+        </is>
+      </c>
     </row>
     <row r="676" hidden="1" ht="16" customHeight="1">
       <c r="A676" s="1" t="inlineStr">
@@ -12663,13 +12810,17 @@
       </c>
       <c r="B678" s="2" t="inlineStr">
         <is>
-          <t>mindspore.set_context</t>
+          <t>mindspore.device_context.ascend.op_tuning.op_compile</t>
         </is>
       </c>
       <c r="C678" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E678" s="2" t="n"/>
+      <c r="E678" s="2" t="inlineStr">
+        <is>
+          <t>set_context(ascend_config={"jit_compile": ...}) 已废弃，最新文档建议使用 ascend.op_tuning.op_compile；需核对 torch_npu set_compile_mode 语义</t>
+        </is>
+      </c>
     </row>
     <row r="679" hidden="1" ht="16" customHeight="1">
       <c r="A679" s="1" t="inlineStr">
@@ -12679,13 +12830,17 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>mindspore.hal.StreamCtx</t>
+          <t>mindspore.runtime.StreamCtx</t>
         </is>
       </c>
       <c r="C679" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E679" s="2" t="n"/>
+      <c r="E679" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="680" hidden="1" ht="16" customHeight="1">
       <c r="A680" s="1" t="inlineStr">
@@ -12695,13 +12850,17 @@
       </c>
       <c r="B680" s="1" t="inlineStr">
         <is>
-          <t>mindspore.hal.synchronize</t>
+          <t>mindspore.runtime.synchronize</t>
         </is>
       </c>
       <c r="C680" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E680" s="2" t="n"/>
+      <c r="E680" s="2" t="inlineStr">
+        <is>
+          <t>hal 接口已废弃，按最新 MindSpore 文档改用 runtime</t>
+        </is>
+      </c>
     </row>
     <row r="681" hidden="1" ht="16" customHeight="1">
       <c r="A681" s="1" t="inlineStr">
@@ -13839,12 +13998,12 @@
       </c>
       <c r="D753" s="2" t="inlineStr">
         <is>
-          <t>hyper_parallel.fully_shard; hyper_parallel.HSDPModule; mindspore.parallel.auto_parallel.AutoParallel.hsdp; mindspore.set_auto_parallel_context(enable_parallel_optimizer=True); mindspore.parallel.distributed.DistributedDataParallel</t>
+          <t>hyper_parallel.fully_shard; hyper_parallel.HSDPModule; mindspore.parallel.auto_parallel.AutoParallel.hsdp; mindspore.parallel.distributed.DistributedDataParallel</t>
         </is>
       </c>
       <c r="E753" s="2" t="inlineStr">
         <is>
-          <t>HyperParallel HSDP是最接近FSDP的外部库替代；MindSpore原生可用自动/半自动并行、优化器并行或DDP，但不是同名等价封装</t>
+          <t>HyperParallel HSDP是最接近FSDP的外部库替代；MindSpore原生可用 AutoParallel/HSDP 或 DDP，但不是同名等价封装；已移除废弃的 set_auto_parallel_context 建议</t>
         </is>
       </c>
     </row>
@@ -14867,6 +15026,16 @@
       <c r="C842" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>mindspore.ops.flash_attention_score</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>参数和 layout 有差异</t>
+        </is>
+      </c>
     </row>
     <row r="843" ht="16" customHeight="1">
       <c r="A843" s="1" t="inlineStr">
@@ -14907,7 +15076,16 @@
       <c r="C846" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D846" s="12" t="n"/>
+      <c r="D846" s="12" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.grouped_matmul; mindspore.ops.auto_generate.grouped_matmul_v2; mindspore.ops.auto_generate.grouped_matmul_v4</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；Ascend 融合算子，参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="847" ht="16" customHeight="1">
       <c r="A847" s="1" t="inlineStr">
@@ -14985,6 +15163,11 @@
           <t>torch_npu.npu_rms_norm</t>
         </is>
       </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>mindspore.ops.rms_norm</t>
+        </is>
+      </c>
       <c r="C853" s="5" t="n">
         <v>1</v>
       </c>
@@ -15008,6 +15191,16 @@
       <c r="C855" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>mindspore.ops.rotary_position_embedding</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>rotary_mul 与 rotary_position_embedding 参数语义不同</t>
+        </is>
+      </c>
     </row>
     <row r="856" hidden="1" ht="16" customHeight="1">
       <c r="A856" s="1" t="inlineStr">
@@ -15015,6 +15208,11 @@
           <t>torch_npu.npu_swiglu</t>
         </is>
       </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>mindspore.ops.swiglu</t>
+        </is>
+      </c>
       <c r="C856" s="5" t="n">
         <v>1</v>
       </c>
@@ -15415,17 +15613,17 @@
           <t>torch.npu.get_device_name</t>
         </is>
       </c>
-      <c r="B889" t="inlineStr">
+      <c r="C889" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D889" t="inlineStr">
         <is>
           <t>mindspore.hal.get_device_name</t>
         </is>
       </c>
-      <c r="C889" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="E889" t="inlineStr">
         <is>
-          <t>MindSpore 文档说明该接口后续将废弃</t>
+          <t>MindSpore 文档说明 hal.get_device_name 后续将废弃，未找到 runtime/device_context 公开对等接口</t>
         </is>
       </c>
     </row>
@@ -15515,32 +15713,149 @@
       </c>
     </row>
     <row r="894" hidden="1" ht="16.8" customHeight="1">
-      <c r="A894" s="1" t="n"/>
-      <c r="C894" s="5" t="n"/>
+      <c r="A894" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="C894" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>mindspore.ops.speed_fusion_attention</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>推理融合注意力公开接口，参数和 layout 需核对</t>
+        </is>
+      </c>
     </row>
     <row r="895" hidden="1" ht="16.8" customHeight="1">
-      <c r="A895" s="1" t="n"/>
-      <c r="C895" s="5" t="n"/>
+      <c r="A895" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_grouped_matmul_finalize_routing</t>
+        </is>
+      </c>
+      <c r="C895" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.grouped_matmul; mindspore.ops.auto_generate.moe_finalize_routing</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；未找到单一对等接口，可拆分替代</t>
+        </is>
+      </c>
     </row>
     <row r="896" hidden="1" ht="16.8" customHeight="1">
-      <c r="A896" s="1" t="n"/>
-      <c r="C896" s="5" t="n"/>
+      <c r="A896" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_distribute_combine_v2</t>
+        </is>
+      </c>
+      <c r="C896" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>mindspore.ops.moe_distribute_combine</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；v2/参数可能不同</t>
+        </is>
+      </c>
     </row>
     <row r="897" hidden="1" ht="16.8" customHeight="1">
-      <c r="A897" s="1" t="n"/>
-      <c r="C897" s="5" t="n"/>
+      <c r="A897" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_distribute_dispatch_v2</t>
+        </is>
+      </c>
+      <c r="C897" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>mindspore.ops.moe_distribute_dispatch</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；v2/参数可能不同</t>
+        </is>
+      </c>
     </row>
     <row r="898" hidden="1" ht="16.8" customHeight="1">
-      <c r="A898" s="1" t="n"/>
-      <c r="C898" s="5" t="n"/>
+      <c r="A898" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_finalize_routing</t>
+        </is>
+      </c>
+      <c r="C898" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.moe_finalize_routing</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="899" hidden="1" ht="16.8" customHeight="1">
-      <c r="A899" s="1" t="n"/>
-      <c r="C899" s="5" t="n"/>
+      <c r="A899" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_gating_top_k</t>
+        </is>
+      </c>
+      <c r="C899" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.moe_gating_top_k_softmax</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；包含 softmax/top-k 语义，参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="900" hidden="1" ht="16.8" customHeight="1">
-      <c r="A900" s="1" t="n"/>
-      <c r="C900" s="5" t="n"/>
+      <c r="A900" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_init_routing_v2</t>
+        </is>
+      </c>
+      <c r="C900" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>mindspore.ops.moe_init_routing_v2</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="901" hidden="1" ht="16.8" customHeight="1">
       <c r="A901" s="1" t="inlineStr">
@@ -15683,12 +15998,12 @@
       </c>
       <c r="D909" t="inlineStr">
         <is>
-          <t>mindspore.hal; mindspore.set_device</t>
+          <t>mindspore.runtime; mindspore.set_device; mindspore.device_context.gpu</t>
         </is>
       </c>
       <c r="E909" t="inlineStr">
         <is>
-          <t>设备运行时模块替代，非一对一等价</t>
+          <t>设备运行时模块替代，非一对一等价；已移除废弃 hal 模块</t>
         </is>
       </c>
     </row>
@@ -15753,12 +16068,12 @@
       </c>
       <c r="D914" t="inlineStr">
         <is>
-          <t>mindspore.get_context("device_target")</t>
+          <t>mindspore.get_current_device</t>
         </is>
       </c>
       <c r="E914" t="inlineStr">
         <is>
-          <t>只能获取 device_target，不是 torch device 对象</t>
+          <t>只能获取当前 MindSpore 设备信息，不是 torch device 对象；原 mindspore.get_context("device_target") 已废弃</t>
         </is>
       </c>
     </row>
@@ -15840,7 +16155,7 @@
       </c>
       <c r="B919" t="inlineStr">
         <is>
-          <t>mindspore.ops.masked_fill</t>
+          <t>mindspore.mint.where</t>
         </is>
       </c>
       <c r="C919" s="5" t="n">
@@ -15849,6 +16164,11 @@
       <c r="D919" t="inlineStr">
         <is>
           <t>mindspore.Tensor.masked_fill</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>mindspore.ops.masked_fill 已废弃，建议改写为 where(mask, value, input)，需处理 value 广播/类型</t>
         </is>
       </c>
     </row>
@@ -15953,12 +16273,12 @@
       </c>
       <c r="D925" t="inlineStr">
         <is>
-          <t>mindspore.hal; mindspore.set_device</t>
+          <t>mindspore.runtime; mindspore.set_device; mindspore.device_context.ascend</t>
         </is>
       </c>
       <c r="E925" t="inlineStr">
         <is>
-          <t>NPU 运行时模块替代，非一对一等价</t>
+          <t>NPU 运行时模块替代，非一对一等价；已移除废弃 hal 模块</t>
         </is>
       </c>
     </row>
@@ -16028,7 +16348,7 @@
       </c>
       <c r="E930" t="inlineStr">
         <is>
-          <t>仅能替代部分设备属性</t>
+          <t>仅能替代部分设备属性；hal 设备属性查询接口后续将废弃，未找到 runtime/device_context 公开对等接口</t>
         </is>
       </c>
     </row>
@@ -16138,13 +16458,18 @@
           <t>torch.npu.mem_get_info</t>
         </is>
       </c>
-      <c r="B936" t="inlineStr">
-        <is>
-          <t>mindspore.hal.mem_get_info</t>
-        </is>
-      </c>
       <c r="C936" s="5" t="n">
         <v>1</v>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>mindspore.runtime.memory_stats; mindspore.runtime.memory_reserved; mindspore.runtime.memory_allocated</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>最新代码/docs 未找到 mindspore.hal.mem_get_info；可用 memory_* 组合近似，非一对一等价</t>
+        </is>
       </c>
     </row>
     <row r="937" hidden="1" ht="16.8" customHeight="1">
@@ -16158,12 +16483,12 @@
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>mindspore.runtime.memory; mindspore.hal</t>
+          <t>mindspore.runtime.memory_stats; mindspore.runtime.memory_reserved; mindspore.runtime.memory_allocated; mindspore.runtime.empty_cache</t>
         </is>
       </c>
       <c r="E937" t="inlineStr">
         <is>
-          <t>运行时内存模块替代，非一对一等价</t>
+          <t>运行时内存接口替代，非一对一等价；已移除废弃 hal 模块</t>
         </is>
       </c>
     </row>
@@ -16303,8 +16628,24 @@
       </c>
     </row>
     <row r="949" hidden="1" ht="16.8" customHeight="1">
-      <c r="A949" s="1" t="n"/>
-      <c r="C949" s="5" t="n"/>
+      <c r="A949" s="1" t="inlineStr">
+        <is>
+          <t>torch.ops.custom.npu_ai_infra_kv_quant_sparse_flash_attention</t>
+        </is>
+      </c>
+      <c r="C949" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>mindspore.ops.sparse_flash_attention</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>自定义接口，KV quant 参数需人工核对</t>
+        </is>
+      </c>
     </row>
     <row r="950" ht="16.8" customHeight="1">
       <c r="A950" s="1" t="inlineStr">
@@ -16327,8 +16668,24 @@
       </c>
     </row>
     <row r="952" hidden="1" ht="16.8" customHeight="1">
-      <c r="A952" s="1" t="n"/>
-      <c r="C952" s="5" t="n"/>
+      <c r="A952" s="1" t="inlineStr">
+        <is>
+          <t>torch.ops.custom.npu_ai_infra_sparse_flash_attention_pioneer</t>
+        </is>
+      </c>
+      <c r="C952" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>mindspore.ops.sparse_flash_attention</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>自定义接口，参数需人工核对</t>
+        </is>
+      </c>
     </row>
     <row r="953" hidden="1" ht="16.8" customHeight="1">
       <c r="A953" s="1" t="inlineStr">
@@ -16371,8 +16728,29 @@
       </c>
     </row>
     <row r="955" hidden="1" ht="16.8" customHeight="1">
-      <c r="A955" s="1" t="n"/>
-      <c r="C955" s="5" t="n"/>
+      <c r="A955" s="1" t="inlineStr">
+        <is>
+          <t>torch.ops.npu.npu_fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="C955" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>mindspore.ops.speed_fusion_attention</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>参数和 layout 需核对</t>
+        </is>
+      </c>
     </row>
     <row r="956" ht="16.8" customHeight="1">
       <c r="A956" s="1" t="inlineStr">
@@ -16485,12 +16863,44 @@
       </c>
     </row>
     <row r="964" hidden="1" ht="16.8" customHeight="1">
-      <c r="A964" s="1" t="n"/>
-      <c r="C964" s="5" t="n"/>
+      <c r="A964" s="1" t="inlineStr">
+        <is>
+          <t>torch.ops.vllm.unified_attention</t>
+        </is>
+      </c>
+      <c r="C964" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score; mindspore.ops.flash_attention_score</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>vLLM 自定义接口，需按注意力场景改写</t>
+        </is>
+      </c>
     </row>
     <row r="965" hidden="1" ht="16.8" customHeight="1">
-      <c r="A965" s="1" t="n"/>
-      <c r="C965" s="5" t="n"/>
+      <c r="A965" s="1" t="inlineStr">
+        <is>
+          <t>torch.ops.vllm.unified_attention_with_output</t>
+        </is>
+      </c>
+      <c r="C965" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score; mindspore.ops.flash_attention_score</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>vLLM 自定义接口，需按注意力场景改写</t>
+        </is>
+      </c>
     </row>
     <row r="966" hidden="1" ht="16.8" customHeight="1">
       <c r="A966" s="1" t="inlineStr">
@@ -17063,12 +17473,39 @@
       </c>
     </row>
     <row r="1006" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1006" s="1" t="n"/>
-      <c r="C1006" s="5" t="n"/>
+      <c r="A1006" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_add_rms_norm</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>mindspore.ops.add_rms_norm</t>
+        </is>
+      </c>
+      <c r="C1006" s="5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="1007" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1007" s="1" t="n"/>
-      <c r="C1007" s="5" t="n"/>
+      <c r="A1007" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_apply_rotary_pos_emb</t>
+        </is>
+      </c>
+      <c r="C1007" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.apply_rotary_pos_emb; mindspore.ops.rotary_position_embedding</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；参数语义需人工核对</t>
+        </is>
+      </c>
     </row>
     <row r="1008" ht="16.8" customHeight="1">
       <c r="A1008" s="1" t="inlineStr">
@@ -17121,20 +17558,99 @@
       </c>
     </row>
     <row r="1012" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1012" s="1" t="n"/>
-      <c r="C1012" s="5" t="n"/>
+      <c r="A1012" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_fused_infer_attention_score.out</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="C1012" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>mindspore.ops.speed_fusion_attention</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>out 变体需改写为普通返回值</t>
+        </is>
+      </c>
     </row>
     <row r="1013" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1013" s="1" t="n"/>
-      <c r="C1013" s="5" t="n"/>
+      <c r="A1013" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_fused_infer_attention_score_v2</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="C1013" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>mindspore.ops.speed_fusion_attention</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>v2 参数和 layout 需核对</t>
+        </is>
+      </c>
     </row>
     <row r="1014" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1014" s="1" t="n"/>
-      <c r="C1014" s="5" t="n"/>
+      <c r="A1014" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_fused_infer_attention_score_v2.out</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="C1014" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>mindspore.ops.speed_fusion_attention</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>out/v2 变体需改写为普通返回值</t>
+        </is>
+      </c>
     </row>
     <row r="1015" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1015" s="1" t="n"/>
-      <c r="C1015" s="5" t="n"/>
+      <c r="A1015" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_interleave_rope</t>
+        </is>
+      </c>
+      <c r="C1015" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>mindspore.ops.rotary_position_embedding</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>rotary/rope 类替代，参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="1016" ht="16.8" customHeight="1">
       <c r="A1016" s="1" t="inlineStr">
@@ -17197,20 +17713,84 @@
       </c>
     </row>
     <row r="1022" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1022" s="1" t="n"/>
-      <c r="C1022" s="5" t="n"/>
+      <c r="A1022" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_compute_expert_tokens</t>
+        </is>
+      </c>
+      <c r="C1022" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.moe_compute_expert_tokens</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="1023" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1023" s="1" t="n"/>
-      <c r="C1023" s="5" t="n"/>
+      <c r="A1023" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_gating_top_k_softmax</t>
+        </is>
+      </c>
+      <c r="C1023" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.moe_gating_top_k_softmax</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="1024" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1024" s="1" t="n"/>
-      <c r="C1024" s="5" t="n"/>
+      <c r="A1024" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_moe_init_routing</t>
+        </is>
+      </c>
+      <c r="C1024" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>mindspore.ops.auto_generate.moe_init_routing; mindspore.ops.moe_init_routing_v2</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>代码已有，未对外；参数不同</t>
+        </is>
+      </c>
     </row>
     <row r="1025" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1025" s="1" t="n"/>
-      <c r="C1025" s="5" t="n"/>
+      <c r="A1025" s="1" t="inlineStr">
+        <is>
+          <t>torch_npu.npu_mrope</t>
+        </is>
+      </c>
+      <c r="C1025" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>mindspore.ops.rotary_position_embedding</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>mrope 需按多模态 rope 语义人工改写</t>
+        </is>
+      </c>
     </row>
     <row r="1026" ht="16.8" customHeight="1">
       <c r="A1026" s="1" t="inlineStr">
@@ -17333,8 +17913,29 @@
       </c>
     </row>
     <row r="1036" hidden="1" ht="16.8" customHeight="1">
-      <c r="A1036" s="1" t="n"/>
-      <c r="C1036" s="5" t="n"/>
+      <c r="A1036" s="1" t="inlineStr">
+        <is>
+          <t>torchair.ops.npu_fused_infer_attention_score_v2</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>mindspore.ops.fused_infer_attention_score</t>
+        </is>
+      </c>
+      <c r="C1036" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>mindspore.ops.speed_fusion_attention</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>torchair 编译后端接口，迁移时改用 MindSpore 原生接口</t>
+        </is>
+      </c>
     </row>
     <row r="1037" ht="16.8" customHeight="1">
       <c r="A1037" s="1" t="inlineStr">

</xml_diff>